<commit_message>
Fix Cross Hierarchy Add New reliability, multi-set Excel parsing, maximized window support, auto run summary
</commit_message>
<xml_diff>
--- a/Test Documentxl.xlsx
+++ b/Test Documentxl.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maheswar.reddy\APP Simulation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B965566D-B2C4-4EA9-8CB4-783959470B6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6569C6DB-485F-485B-A3BB-32941379DE90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{61D4B329-8650-4C66-857D-4CE8D903A61D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{61D4B329-8650-4C66-857D-4CE8D903A61D}"/>
   </bookViews>
   <sheets>
     <sheet name="Credentials" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="87">
   <si>
     <t>app_username</t>
   </si>
@@ -211,6 +211,94 @@
   </si>
   <si>
     <t>Placeholder_Location_5</t>
+  </si>
+  <si>
+    <t>Cross Hierarchy</t>
+  </si>
+  <si>
+    <t>MFG_SITE_ID</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>POS_SITE_ID</t>
+  </si>
+  <si>
+    <t>POS_ORDER_TYPE</t>
+  </si>
+  <si>
+    <t>CUSTOMER_PART_NO</t>
+  </si>
+  <si>
+    <t>MFG_ORDER_TYPE</t>
+  </si>
+  <si>
+    <t>PRIMARY_MFG_SITE</t>
+  </si>
+  <si>
+    <t>MANUFACTURING_OFFSET</t>
+  </si>
+  <si>
+    <t>BOOKINGS_OFFSET</t>
+  </si>
+  <si>
+    <t>PCS_IS_DISCONTINUED</t>
+  </si>
+  <si>
+    <t>Hierarchy 1
+Product</t>
+  </si>
+  <si>
+    <t>Hierarchy 2 Channel</t>
+  </si>
+  <si>
+    <t>Hierarchy Location</t>
+  </si>
+  <si>
+    <t>ITEM</t>
+  </si>
+  <si>
+    <t>Level1</t>
+  </si>
+  <si>
+    <t>Level2</t>
+  </si>
+  <si>
+    <t>Mapped Column</t>
+  </si>
+  <si>
+    <t>MFG_SITE_ID_A</t>
+  </si>
+  <si>
+    <t>POS_SITE_ID_A</t>
+  </si>
+  <si>
+    <t>POS_ORDER_TYPE_A</t>
+  </si>
+  <si>
+    <t>CUSTOMER_PART_NO_A</t>
+  </si>
+  <si>
+    <t>MFG_ORDER_TYPE_A</t>
+  </si>
+  <si>
+    <t>PRIMARY_MFG_SITE_A</t>
+  </si>
+  <si>
+    <t>MANUFACTURING_OFFSET_A</t>
+  </si>
+  <si>
+    <t>BOOKINGS_OFFSET_A</t>
+  </si>
+  <si>
+    <t>PCS_IS_DISCONTINUED_A</t>
+  </si>
+  <si>
+    <t>set 1</t>
+  </si>
+  <si>
+    <t>set2</t>
   </si>
 </sst>
 </file>
@@ -222,7 +310,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy;@"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -270,6 +358,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -309,7 +403,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="45">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
@@ -361,19 +455,35 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="47" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="47" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="45">
+  <cellStyles count="49">
     <cellStyle name="Comma 2" xfId="8" xr:uid="{207A94A0-39A6-4518-B6FF-043DF01B5F29}"/>
     <cellStyle name="Comma 3" xfId="12" xr:uid="{1B733330-AAF3-43FE-9959-FE1DC4C8D083}"/>
     <cellStyle name="Comma 4" xfId="4" xr:uid="{7571162E-B3DA-42BC-AE64-4DECDD98CA1C}"/>
@@ -404,6 +514,10 @@
     <cellStyle name="Normal 2 2 2 3 4" xfId="24" xr:uid="{73B2FE84-DBBB-4455-9A7F-2D926767E24B}"/>
     <cellStyle name="Normal 20" xfId="1" xr:uid="{A9BFF64A-BB74-49FF-9538-C694F05FDD19}"/>
     <cellStyle name="Normal 21" xfId="2" xr:uid="{A24CDDC4-DD46-4261-8E2A-AA82D501DA2D}"/>
+    <cellStyle name="Normal 22" xfId="47" xr:uid="{EC1E8DDE-1EC5-4366-B676-A0D70349BDC2}"/>
+    <cellStyle name="Normal 23" xfId="45" xr:uid="{4D2BF18F-05D0-4FF0-B4F5-9F9EDD741375}"/>
+    <cellStyle name="Normal 24" xfId="48" xr:uid="{5830AC7A-62B7-4497-95FD-596BF8E1E218}"/>
+    <cellStyle name="Normal 25" xfId="46" xr:uid="{CEE2BE83-E4BA-4864-B4D0-6C6333C796BC}"/>
     <cellStyle name="Normal 3" xfId="7" xr:uid="{65170AE0-EE29-45FC-83BD-64C18A7AF58D}"/>
     <cellStyle name="Normal 3 2" xfId="23" xr:uid="{41ECF9BD-1A5A-4285-BC4B-EB6029ADD722}"/>
     <cellStyle name="Normal 4" xfId="10" xr:uid="{5697FE90-DC16-49E5-9BA3-BD7F36DE26B9}"/>
@@ -794,14 +908,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17B1ACE0-294C-4A4E-B938-BA67A9EFE7FB}">
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -815,51 +931,53 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -869,60 +987,62 @@
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="A11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="A13" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="A14" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="A15" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>22</v>
       </c>
@@ -938,8 +1058,9 @@
       <c r="E20" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F20" s="6"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>23</v>
       </c>
@@ -947,12 +1068,13 @@
         <v>24</v>
       </c>
       <c r="C21" s="1"/>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="5" t="s">
         <v>34</v>
       </c>
       <c r="E21" s="1"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F21" s="6"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>39</v>
       </c>
@@ -960,12 +1082,13 @@
         <v>24</v>
       </c>
       <c r="C22" s="1"/>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="5" t="s">
         <v>34</v>
       </c>
       <c r="E22" s="1"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F22" s="6"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>25</v>
       </c>
@@ -973,12 +1096,13 @@
         <v>24</v>
       </c>
       <c r="C23" s="1"/>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="5" t="s">
         <v>34</v>
       </c>
       <c r="E23" s="1"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F23" s="6"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>40</v>
       </c>
@@ -986,14 +1110,15 @@
         <v>24</v>
       </c>
       <c r="C24" s="1"/>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="5" t="s">
         <v>34</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F24" s="6"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>41</v>
       </c>
@@ -1001,14 +1126,15 @@
         <v>24</v>
       </c>
       <c r="C25" s="1"/>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="5" t="s">
         <v>34</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F25" s="6"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>26</v>
       </c>
@@ -1016,12 +1142,13 @@
         <v>24</v>
       </c>
       <c r="C26" s="1"/>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="5" t="s">
         <v>35</v>
       </c>
       <c r="E26" s="1"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F26" s="6"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>42</v>
       </c>
@@ -1029,12 +1156,13 @@
         <v>24</v>
       </c>
       <c r="C27" s="1"/>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="5" t="s">
         <v>34</v>
       </c>
       <c r="E27" s="1"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F27" s="6"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>43</v>
       </c>
@@ -1042,12 +1170,13 @@
         <v>24</v>
       </c>
       <c r="C28" s="1"/>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="5" t="s">
         <v>36</v>
       </c>
       <c r="E28" s="1"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F28" s="6"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>44</v>
       </c>
@@ -1055,12 +1184,13 @@
         <v>24</v>
       </c>
       <c r="C29" s="1"/>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="5" t="s">
         <v>37</v>
       </c>
       <c r="E29" s="1"/>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F29" s="6"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>45</v>
       </c>
@@ -1068,12 +1198,13 @@
         <v>24</v>
       </c>
       <c r="C30" s="1"/>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="5" t="s">
         <v>37</v>
       </c>
       <c r="E30" s="1"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F30" s="6"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>46</v>
       </c>
@@ -1081,12 +1212,13 @@
         <v>24</v>
       </c>
       <c r="C31" s="1"/>
-      <c r="D31" s="4" t="s">
+      <c r="D31" s="5" t="s">
         <v>34</v>
       </c>
       <c r="E31" s="1"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F31" s="6"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>47</v>
       </c>
@@ -1094,12 +1226,13 @@
         <v>24</v>
       </c>
       <c r="C32" s="1"/>
-      <c r="D32" s="4" t="s">
+      <c r="D32" s="5" t="s">
         <v>34</v>
       </c>
       <c r="E32" s="1"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F32" s="6"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>27</v>
       </c>
@@ -1107,12 +1240,13 @@
         <v>13</v>
       </c>
       <c r="C33" s="1"/>
-      <c r="D33" s="4" t="s">
+      <c r="D33" s="5" t="s">
         <v>34</v>
       </c>
       <c r="E33" s="1"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F33" s="6"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>28</v>
       </c>
@@ -1120,12 +1254,13 @@
         <v>13</v>
       </c>
       <c r="C34" s="1"/>
-      <c r="D34" s="4" t="s">
+      <c r="D34" s="5" t="s">
         <v>34</v>
       </c>
       <c r="E34" s="1"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F34" s="6"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>29</v>
       </c>
@@ -1133,12 +1268,13 @@
         <v>13</v>
       </c>
       <c r="C35" s="1"/>
-      <c r="D35" s="4" t="s">
+      <c r="D35" s="5" t="s">
         <v>35</v>
       </c>
       <c r="E35" s="1"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F35" s="6"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>48</v>
       </c>
@@ -1146,12 +1282,13 @@
         <v>13</v>
       </c>
       <c r="C36" s="1"/>
-      <c r="D36" s="4" t="s">
+      <c r="D36" s="5" t="s">
         <v>36</v>
       </c>
       <c r="E36" s="1"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F36" s="6"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>49</v>
       </c>
@@ -1159,12 +1296,13 @@
         <v>13</v>
       </c>
       <c r="C37" s="1"/>
-      <c r="D37" s="4" t="s">
+      <c r="D37" s="5" t="s">
         <v>37</v>
       </c>
       <c r="E37" s="1"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F37" s="6"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>50</v>
       </c>
@@ -1172,12 +1310,13 @@
         <v>13</v>
       </c>
       <c r="C38" s="1"/>
-      <c r="D38" s="4" t="s">
+      <c r="D38" s="5" t="s">
         <v>37</v>
       </c>
       <c r="E38" s="1"/>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F38" s="6"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>51</v>
       </c>
@@ -1185,12 +1324,13 @@
         <v>13</v>
       </c>
       <c r="C39" s="1"/>
-      <c r="D39" s="4" t="s">
+      <c r="D39" s="5" t="s">
         <v>34</v>
       </c>
       <c r="E39" s="1"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F39" s="6"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>52</v>
       </c>
@@ -1198,12 +1338,13 @@
         <v>13</v>
       </c>
       <c r="C40" s="1"/>
-      <c r="D40" s="4" t="s">
+      <c r="D40" s="5" t="s">
         <v>34</v>
       </c>
       <c r="E40" s="1"/>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F40" s="6"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>30</v>
       </c>
@@ -1211,12 +1352,13 @@
         <v>11</v>
       </c>
       <c r="C41" s="1"/>
-      <c r="D41" s="4" t="s">
+      <c r="D41" s="5" t="s">
         <v>35</v>
       </c>
       <c r="E41" s="1"/>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F41" s="6"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>53</v>
       </c>
@@ -1224,12 +1366,13 @@
         <v>11</v>
       </c>
       <c r="C42" s="1"/>
-      <c r="D42" s="4" t="s">
+      <c r="D42" s="5" t="s">
         <v>36</v>
       </c>
       <c r="E42" s="1"/>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F42" s="6"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>54</v>
       </c>
@@ -1237,12 +1380,13 @@
         <v>11</v>
       </c>
       <c r="C43" s="1"/>
-      <c r="D43" s="4" t="s">
+      <c r="D43" s="5" t="s">
         <v>37</v>
       </c>
       <c r="E43" s="1"/>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F43" s="6"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>55</v>
       </c>
@@ -1250,12 +1394,13 @@
         <v>11</v>
       </c>
       <c r="C44" s="1"/>
-      <c r="D44" s="4" t="s">
+      <c r="D44" s="5" t="s">
         <v>37</v>
       </c>
       <c r="E44" s="1"/>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F44" s="6"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>56</v>
       </c>
@@ -1263,12 +1408,13 @@
         <v>11</v>
       </c>
       <c r="C45" s="1"/>
-      <c r="D45" s="4" t="s">
+      <c r="D45" s="5" t="s">
         <v>34</v>
       </c>
       <c r="E45" s="1"/>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F45" s="6"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>57</v>
       </c>
@@ -1276,12 +1422,485 @@
         <v>11</v>
       </c>
       <c r="C46" s="1"/>
-      <c r="D46" s="4" t="s">
+      <c r="D46" s="5" t="s">
         <v>34</v>
       </c>
       <c r="E46" s="1"/>
+      <c r="F46" s="6"/>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G51" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H51" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B52" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E52" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F52" s="5"/>
+      <c r="G52" s="8"/>
+      <c r="H52" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C53" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E53" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F53" s="5"/>
+      <c r="G53" s="8"/>
+      <c r="H53" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B54" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C54" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D54" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E54" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F54" s="5"/>
+      <c r="G54" s="8"/>
+      <c r="H54" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B55" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C55" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D55" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E55" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="F55" s="5"/>
+      <c r="G55" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H55" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B56" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C56" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E56" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F56" s="5"/>
+      <c r="G56" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H56" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="B57" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C57" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D57" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E57" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F57" s="5"/>
+      <c r="G57" s="8"/>
+      <c r="H57" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B58" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D58" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E58" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F58" s="5"/>
+      <c r="G58" s="8"/>
+      <c r="H58" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B59" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C59" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D59" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F59" s="5"/>
+      <c r="G59" s="8"/>
+      <c r="H59" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B60" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D60" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F60" s="5"/>
+      <c r="G60" s="8"/>
+      <c r="H60" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A63" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G63" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H63" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A64" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B64" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C64" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D64" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E64" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F64" s="5"/>
+      <c r="G64" s="8"/>
+      <c r="H64" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A65" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B65" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C65" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D65" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E65" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F65" s="5"/>
+      <c r="G65" s="8"/>
+      <c r="H65" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B66" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C66" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D66" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E66" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F66" s="5"/>
+      <c r="G66" s="8"/>
+      <c r="H66" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B67" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C67" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D67" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E67" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="F67" s="5"/>
+      <c r="G67" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H67" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A68" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="B68" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C68" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D68" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E68" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F68" s="5"/>
+      <c r="G68" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H68" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A69" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="B69" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C69" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D69" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E69" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F69" s="5"/>
+      <c r="G69" s="8"/>
+      <c r="H69" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A70" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B70" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C70" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D70" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F70" s="5"/>
+      <c r="G70" s="8"/>
+      <c r="H70" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A71" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B71" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C71" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D71" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E71" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F71" s="5"/>
+      <c r="G71" s="8"/>
+      <c r="H71" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A72" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="B72" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C72" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D72" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E72" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F72" s="5"/>
+      <c r="G72" s="8"/>
+      <c r="H72" s="8" t="s">
+        <v>60</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>